<commit_message>
Replace project with updated version
</commit_message>
<xml_diff>
--- a/next_week_weights_estimate_app.xlsx
+++ b/next_week_weights_estimate_app.xlsx
@@ -464,19 +464,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1.81285514432328e-09</v>
+        <v>6.426582659000449e-10</v>
       </c>
       <c r="C2" t="n">
-        <v>1.184464077636434e-09</v>
+        <v>3.206696303476659e-09</v>
       </c>
       <c r="D2" t="n">
-        <v>1.864478199970915e-09</v>
+        <v>6.005419133132101e-10</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9999999951382343</v>
+        <v>0.9999999955501311</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46080</v>
+        <v>46087</v>
       </c>
     </row>
   </sheetData>

</xml_diff>